<commit_message>
Actualizacion automatica del mapa (2026-06-01 11:48:12)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Fiberwork.xlsx
+++ b/mapa_interactivo_Fiberwork.xlsx
@@ -8085,7 +8085,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>814105603</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
@@ -8171,7 +8171,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>814107131</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
@@ -10837,7 +10837,7 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>GENERADOR DE OT NO ENCUENTRA DIRECCION</t>
+          <t>814105853</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
@@ -11439,7 +11439,7 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>GENERADOR DE OT NO ENCUENTRA DIRECCION</t>
+          <t>814105864</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
@@ -12801,7 +12801,11 @@
           <t>FIBERWORK</t>
         </is>
       </c>
-      <c r="G145" t="inlineStr"/>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>814108068</t>
+        </is>
+      </c>
       <c r="H145" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -12965,7 +12969,11 @@
           <t>FIBERWORK</t>
         </is>
       </c>
-      <c r="G147" t="inlineStr"/>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>814108086</t>
+        </is>
+      </c>
       <c r="H147" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-06-01 13:06:09)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Fiberwork.xlsx
+++ b/mapa_interactivo_Fiberwork.xlsx
@@ -8515,7 +8515,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>814109847</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
@@ -12637,7 +12637,11 @@
           <t>FIBERWORK</t>
         </is>
       </c>
-      <c r="G143" t="inlineStr"/>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>814109709</t>
+        </is>
+      </c>
       <c r="H143" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -12719,7 +12723,11 @@
           <t>FIBERWORK</t>
         </is>
       </c>
-      <c r="G144" t="inlineStr"/>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>814109753</t>
+        </is>
+      </c>
       <c r="H144" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-06-02 15:37:55)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Fiberwork.xlsx
+++ b/mapa_interactivo_Fiberwork.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R148"/>
+  <dimension ref="A1:R154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,17 +439,17 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>OT</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Proveedor Asignado</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>OT</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
@@ -531,17 +531,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>798385574</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>FIBERWORK</t>
-        </is>
-      </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>798385574</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -617,17 +617,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>798513095</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>FIBERWORK</t>
-        </is>
-      </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>798513095</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -699,17 +699,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>798894281</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>798894281</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -785,17 +785,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>789151020</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>789151020</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -871,17 +871,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t>802438793</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>FIBERWORK</t>
-        </is>
-      </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>802438793</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -957,17 +957,17 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
+          <t>802774521</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>FIBERWORK</t>
-        </is>
-      </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>802774521</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1043,17 +1043,17 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>803039902</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>803039902</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1129,17 +1129,17 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>803666441</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>803666441</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1215,17 +1215,17 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>804161204</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>804161204</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1301,17 +1301,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>804161231</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>804161231</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1387,17 +1387,17 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>804270064</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>804270064</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1473,17 +1473,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>804270068</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>804270068</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1559,17 +1559,17 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>804270074</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>804270074</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1645,17 +1645,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>804569065</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>804569065</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1731,17 +1731,17 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
+          <t>804903806</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>FIBERWORK</t>
-        </is>
-      </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>804903806</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1817,17 +1817,17 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
+          <t>805507294</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>FIBERWORK</t>
-        </is>
-      </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>805507294</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1903,17 +1903,17 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
+          <t>805579188</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>FIBERWORK</t>
-        </is>
-      </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>805579188</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1989,17 +1989,17 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>806926385</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>806926385</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -2075,17 +2075,17 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>806926861</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>806926861</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -2161,17 +2161,17 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>807187860</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>807187860</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -2247,17 +2247,17 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
+          <t>807215439</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>FIBERWORK</t>
-        </is>
-      </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>807215439</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2333,17 +2333,17 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>807215458</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>807215458</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2419,17 +2419,17 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810533286</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>810533286</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -2505,17 +2505,17 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
+          <t>ICD31456940</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>FIBERWORK</t>
-        </is>
-      </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>ICD31456940</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H25" t="inlineStr"/>
@@ -2587,17 +2587,17 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
+          <t>807851584</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>FIBERWORK</t>
-        </is>
-      </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>807851584</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H26" t="inlineStr"/>
@@ -2669,17 +2669,17 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>808194254</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>808194254</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2755,17 +2755,17 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>808194260</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>808194260</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2841,17 +2841,17 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>808373657</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>808373657</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -2927,17 +2927,17 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>808579773</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>808579773</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -3013,17 +3013,17 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>808703866</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>808703866</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -3099,17 +3099,17 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
+          <t>808918687</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>FIBERWORK</t>
-        </is>
-      </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>808918687</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -3185,17 +3185,17 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>809195660</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>809195660</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -3271,17 +3271,17 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>809195664</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>809195664</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -3357,17 +3357,17 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>809732190</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>809732190</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -3443,17 +3443,17 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>809800215</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>809800215</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -3529,17 +3529,17 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>809910086</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>809910086</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -3615,17 +3615,17 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>809979740</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>809979740</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -3701,17 +3701,17 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810093628</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>810093628</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -3787,17 +3787,17 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810244454</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>810244454</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -3873,17 +3873,17 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810244458</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>810244458</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -3959,17 +3959,17 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>ICD31464881</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>ICD31464881</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -4045,17 +4045,17 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810394752</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>810394752</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -4131,17 +4131,17 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810398934</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>810398934</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -4217,17 +4217,17 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810416656</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>810416656</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -4303,17 +4303,17 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810451584</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>810451584</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -4389,17 +4389,17 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810487023</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>810487023</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -4475,17 +4475,17 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810487035</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>810487035</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -4561,17 +4561,17 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810712796</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>810712796</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -4647,17 +4647,17 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810787612</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>810787612</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -4733,17 +4733,17 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810787513</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>810787513</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -4819,17 +4819,17 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810804303</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>810804303</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -4905,17 +4905,17 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810804462</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>810804462</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -4991,17 +4991,17 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810804451</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>810804451</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -5077,17 +5077,17 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810804383</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>810804383</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -5163,17 +5163,17 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t xml:space="preserve">01503983 </t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t xml:space="preserve">01503983 </t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -5249,17 +5249,17 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810804369</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>810804369</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -5335,17 +5335,17 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810820592</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>810820592</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -5421,17 +5421,17 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810862729</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>810862729</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -5507,17 +5507,17 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810984598</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>810984598</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -5593,17 +5593,17 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810984700</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>810984700</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -5679,17 +5679,17 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811198737</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>811198737</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -5765,17 +5765,17 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811198696</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>811198696</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -5851,17 +5851,17 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811198676</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>811198676</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -5937,17 +5937,17 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>02013924</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>02013924</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -6023,17 +6023,17 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811299416</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>811299416</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -6109,17 +6109,17 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811299443</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>811299443</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -6195,17 +6195,17 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
+          <t>811453866</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>FIBERWORK</t>
-        </is>
-      </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>811453866</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -6281,17 +6281,17 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811453904</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>811453904</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -6367,17 +6367,17 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t xml:space="preserve">02511385 </t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t xml:space="preserve">02511385 </t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -6453,17 +6453,17 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811454440</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>811454440</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -6539,17 +6539,17 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811454538</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>811454538</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -6625,17 +6625,17 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t>FIBERWORK</t>
-        </is>
-      </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -6699,17 +6699,17 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812439895</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>812439895</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -6785,17 +6785,17 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811626888</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>811626888</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -6871,17 +6871,17 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811626986</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>811626986</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -6957,17 +6957,17 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811626981</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>811626981</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -7043,17 +7043,17 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811627014</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>811627014</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -7129,17 +7129,17 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811627077</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>811627077</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -7215,17 +7215,17 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811627062</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>811627062</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -7301,17 +7301,17 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811627128</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>811627128</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -7387,17 +7387,17 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812439968</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>812439968</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -7473,17 +7473,17 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812440156</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>812440156</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -7559,17 +7559,17 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812440173</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>812440173</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -7645,17 +7645,17 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812440165</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>812440165</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
@@ -7731,17 +7731,17 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812440614</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>812440614</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -7817,17 +7817,17 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812440354</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>812440354</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -7903,17 +7903,17 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812440282</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>812440282</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
@@ -7989,17 +7989,17 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812503638</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>812503638</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
@@ -8075,17 +8075,17 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814105603</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>814105603</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
@@ -8161,17 +8161,17 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814107131</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>814107131</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
@@ -8247,17 +8247,17 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812879940</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>812879940</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
@@ -8333,17 +8333,17 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812879982</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>812879982</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
@@ -8419,17 +8419,17 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812880406</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>812880406</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
@@ -8505,17 +8505,17 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814109847</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>814109847</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
@@ -8591,17 +8591,17 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812880625</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>812880625</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
@@ -8677,17 +8677,17 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812880655</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>812880655</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
@@ -8763,17 +8763,17 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812880662</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>812880662</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
@@ -8849,17 +8849,17 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812880685</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>812880685</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
@@ -8935,17 +8935,17 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812880736</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>812880736</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
@@ -9021,17 +9021,17 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813046342</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>813046342</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
@@ -9107,17 +9107,17 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813046658</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>813046658</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
@@ -9193,17 +9193,17 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813046791</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>813046791</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
@@ -9279,17 +9279,17 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813046795</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>813046795</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
@@ -9365,17 +9365,17 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813046806</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>813046806</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
@@ -9451,17 +9451,17 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813046819</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>813046819</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
@@ -9537,17 +9537,17 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813046866</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>813046866</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
@@ -9623,17 +9623,17 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813046970</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>813046970</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
@@ -9709,17 +9709,17 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813046971</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>813046971</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
@@ -9795,17 +9795,17 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813046994</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>813046994</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
@@ -9881,17 +9881,17 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813047007</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>813047007</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
@@ -9967,17 +9967,17 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813047012</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>813047012</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
@@ -10053,17 +10053,17 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813047017</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>813047017</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
@@ -10139,17 +10139,17 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813047019</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>813047019</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
@@ -10225,17 +10225,17 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813047657</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>813047657</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
@@ -10311,17 +10311,17 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813304903</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>813304903</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
@@ -10397,17 +10397,17 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813304915</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>813304915</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
@@ -10483,17 +10483,17 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813350607</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>813350607</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
@@ -10569,17 +10569,17 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813350620</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>813350620</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
@@ -10655,17 +10655,17 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813350953</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>813350953</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
@@ -10741,17 +10741,17 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813351576</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>813351576</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
@@ -10827,17 +10827,17 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814105853</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>814105853</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
@@ -10913,17 +10913,17 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813352212</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>813352212</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
@@ -10999,17 +10999,17 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813352473</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>813352473</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
@@ -11085,17 +11085,17 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813352481</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>813352481</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
@@ -11171,17 +11171,17 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813352482</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>813352482</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
@@ -11257,17 +11257,17 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813352486</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>813352486</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
@@ -11343,17 +11343,17 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813352494</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>813352494</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
@@ -11429,17 +11429,17 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814105864</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>814105864</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
@@ -11515,17 +11515,17 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813352497</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>813352497</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
@@ -11601,17 +11601,17 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813352774</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>813352774</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
@@ -11687,17 +11687,17 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813352855</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>813352855</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
@@ -11773,17 +11773,17 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813352873</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>813352873</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
@@ -11859,17 +11859,17 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813353299</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>813353299</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
@@ -11945,17 +11945,17 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813631423</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>813631423</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
@@ -12031,17 +12031,17 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813631424</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>813631424</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
@@ -12117,17 +12117,17 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813631550</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>813631550</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
@@ -12203,17 +12203,17 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813632251</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>813632251</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
@@ -12289,17 +12289,17 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813632257</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>813632257</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
@@ -12375,17 +12375,17 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813632439</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>813632439</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
@@ -12459,17 +12459,17 @@
           <t>5</t>
         </is>
       </c>
-      <c r="E141" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+      <c r="E141" t="inlineStr"/>
       <c r="F141" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
-        </is>
-      </c>
-      <c r="G141" t="inlineStr"/>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>FIBERWORK</t>
+        </is>
+      </c>
       <c r="H141" t="inlineStr">
         <is>
           <t>NORMALIZAR RIENDA A PIQUE</t>
@@ -12543,17 +12543,17 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813352547</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>813352547</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
@@ -12629,17 +12629,17 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814109709</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>814109709</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
@@ -12715,17 +12715,17 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814109753</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>814109753</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
@@ -12801,17 +12801,17 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814108068</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>814108068</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
@@ -12885,17 +12885,17 @@
           <t>3</t>
         </is>
       </c>
-      <c r="E146" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+      <c r="E146" t="inlineStr"/>
       <c r="F146" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
-        </is>
-      </c>
-      <c r="G146" t="inlineStr"/>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>FIBERWORK</t>
+        </is>
+      </c>
       <c r="H146" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -12969,17 +12969,17 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814108086</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>814108086</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
@@ -13055,15 +13055,19 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814111727</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
-        </is>
-      </c>
-      <c r="G148" t="inlineStr"/>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>FIBERWORK</t>
+        </is>
+      </c>
       <c r="H148" t="inlineStr">
         <is>
           <t>COLUMNA INCLINADA</t>
@@ -13071,7 +13075,7 @@
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J148" t="inlineStr">
@@ -13111,6 +13115,522 @@
       <c r="R148" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>-776</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>6/2/2026</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>ALSINA, ADOLFO 2457</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>814125554</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>FIBERWORK</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>base corroida</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L149" t="n">
+        <v>1</v>
+      </c>
+      <c r="M149" t="n">
+        <v>-58.401052</v>
+      </c>
+      <c r="N149" t="n">
+        <v>-34.612103</v>
+      </c>
+      <c r="O149" t="inlineStr">
+        <is>
+          <t>Almagro</t>
+        </is>
+      </c>
+      <c r="P149" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q149" t="inlineStr">
+        <is>
+          <t>CEN-H</t>
+        </is>
+      </c>
+      <c r="R149" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>-801</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>6/2/2026</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>YRIGOYEN, HIPOLITO 2754</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>814125643</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>FIBERWORK</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>base corroida</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L150" t="n">
+        <v>1</v>
+      </c>
+      <c r="M150" t="n">
+        <v>-58.405116</v>
+      </c>
+      <c r="N150" t="n">
+        <v>-34.611253</v>
+      </c>
+      <c r="O150" t="inlineStr">
+        <is>
+          <t>Almagro</t>
+        </is>
+      </c>
+      <c r="P150" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q150" t="inlineStr">
+        <is>
+          <t>CEN-H</t>
+        </is>
+      </c>
+      <c r="R150" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>-810</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>6/2/2026</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>MEXICO 2183</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>814125664</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>FIBERWORK</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>base corroida</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L151" t="n">
+        <v>1</v>
+      </c>
+      <c r="M151" t="n">
+        <v>-58.397489</v>
+      </c>
+      <c r="N151" t="n">
+        <v>-34.616089</v>
+      </c>
+      <c r="O151" t="inlineStr">
+        <is>
+          <t>Almagro</t>
+        </is>
+      </c>
+      <c r="P151" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q151" t="inlineStr">
+        <is>
+          <t>CEN-C</t>
+        </is>
+      </c>
+      <c r="R151" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>-818</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>6/2/2026</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>PRINGLES 795</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>814125690</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>FIBERWORK</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>base podrida</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L152" t="n">
+        <v>1</v>
+      </c>
+      <c r="M152" t="n">
+        <v>-58.427096</v>
+      </c>
+      <c r="N152" t="n">
+        <v>-34.602833</v>
+      </c>
+      <c r="O152" t="inlineStr">
+        <is>
+          <t>Almagro</t>
+        </is>
+      </c>
+      <c r="P152" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q152" t="inlineStr">
+        <is>
+          <t>CLI-M</t>
+        </is>
+      </c>
+      <c r="R152" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>-820</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>6/2/2026</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>RIOBAMBA 558</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>814125697</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>FIBERWORK</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>base corroida</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L153" t="n">
+        <v>1</v>
+      </c>
+      <c r="M153" t="n">
+        <v>-58.394106</v>
+      </c>
+      <c r="N153" t="n">
+        <v>-34.602514</v>
+      </c>
+      <c r="O153" t="inlineStr">
+        <is>
+          <t>Almagro</t>
+        </is>
+      </c>
+      <c r="P153" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q153" t="inlineStr">
+        <is>
+          <t>RET-J</t>
+        </is>
+      </c>
+      <c r="R153" t="inlineStr">
+        <is>
+          <t>ARATO-25058.PO.1RET</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>-828</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>6/2/2026</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>TUCUMAN 2074</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>FIBERWORK</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>base corroida</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>Nodo Teco</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L154" t="n">
+        <v>1</v>
+      </c>
+      <c r="M154" t="n">
+        <v>-58.396631</v>
+      </c>
+      <c r="N154" t="n">
+        <v>-34.60222</v>
+      </c>
+      <c r="O154" t="inlineStr">
+        <is>
+          <t>Almagro</t>
+        </is>
+      </c>
+      <c r="P154" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q154" t="inlineStr">
+        <is>
+          <t>RET-J</t>
+        </is>
+      </c>
+      <c r="R154" t="inlineStr">
+        <is>
+          <t>ARATO-25058.PO.1RET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-06-11 11:03:19)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Fiberwork.xlsx
+++ b/mapa_interactivo_Fiberwork.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R152"/>
+  <dimension ref="A1:R151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8657,17 +8657,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>8265</t>
+          <t>8703</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>3/23/2026</t>
+          <t>3/28/2026</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>HUMBERTO 1 1999</t>
+          <t>RIVADAVIA AV 1985</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -8682,7 +8682,7 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>812880685</t>
+          <t>812880736</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
@@ -8692,12 +8692,12 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>APLOMAR COLUMNA</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
@@ -8714,14 +8714,14 @@
         <v>1</v>
       </c>
       <c r="M97" t="n">
-        <v>-58.394304</v>
+        <v>-58.394609</v>
       </c>
       <c r="N97" t="n">
-        <v>-34.621645</v>
+        <v>-34.609304</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P97" t="inlineStr">
@@ -8731,7 +8731,7 @@
       </c>
       <c r="Q97" t="inlineStr">
         <is>
-          <t>CEN-B</t>
+          <t>CLI-B</t>
         </is>
       </c>
       <c r="R97" t="inlineStr">
@@ -8743,22 +8743,22 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>8703</t>
+          <t>M881</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>3/28/2026</t>
+          <t>4/1/2026</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>RIVADAVIA AV 1985</t>
+          <t>AV LA PLATA 2288</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -8768,7 +8768,7 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>812880736</t>
+          <t>813046342</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
@@ -8778,17 +8778,17 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>APLOMAR COLUMNA</t>
+          <t>DESMONTAR COLUMNA Y  DESPLAZAR PCALOGERO</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -8800,14 +8800,14 @@
         <v>1</v>
       </c>
       <c r="M98" t="n">
-        <v>-58.394609</v>
+        <v>-58.423203</v>
       </c>
       <c r="N98" t="n">
-        <v>-34.609304</v>
+        <v>-34.640909</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P98" t="inlineStr">
@@ -8817,7 +8817,7 @@
       </c>
       <c r="Q98" t="inlineStr">
         <is>
-          <t>CLI-B</t>
+          <t>PPT-L</t>
         </is>
       </c>
       <c r="R98" t="inlineStr">
@@ -8829,22 +8829,22 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>M881</t>
+          <t>8802</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>4/1/2026</t>
+          <t>4/11/2026</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>AV LA PLATA 2288</t>
+          <t>RINCON 731</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -8854,7 +8854,7 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>813046342</t>
+          <t>813046658</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>DESMONTAR COLUMNA Y  DESPLAZAR PCALOGERO</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -8886,14 +8886,14 @@
         <v>1</v>
       </c>
       <c r="M99" t="n">
-        <v>-58.423203</v>
+        <v>-58.396088</v>
       </c>
       <c r="N99" t="n">
-        <v>-34.640909</v>
+        <v>-34.617527</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P99" t="inlineStr">
@@ -8903,7 +8903,7 @@
       </c>
       <c r="Q99" t="inlineStr">
         <is>
-          <t>PPT-L</t>
+          <t>CEN-C</t>
         </is>
       </c>
       <c r="R99" t="inlineStr">
@@ -8915,7 +8915,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>8802</t>
+          <t>S00374917</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -8925,7 +8925,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>RINCON 731</t>
+          <t>24 DE NOVIEMBRE 695</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -8940,7 +8940,7 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>813046658</t>
+          <t>813046791</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
@@ -8972,10 +8972,10 @@
         <v>1</v>
       </c>
       <c r="M100" t="n">
-        <v>-58.396088</v>
+        <v>-58.411053</v>
       </c>
       <c r="N100" t="n">
-        <v>-34.617527</v>
+        <v>-34.618979</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -8989,7 +8989,7 @@
       </c>
       <c r="Q100" t="inlineStr">
         <is>
-          <t>CEN-C</t>
+          <t>CEN-J</t>
         </is>
       </c>
       <c r="R100" t="inlineStr">
@@ -9001,7 +9001,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>S00374917</t>
+          <t>S00379764</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -9011,7 +9011,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>24 DE NOVIEMBRE 695</t>
+          <t>JAURES JEAN 491</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -9026,7 +9026,7 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>813046791</t>
+          <t>813046795</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
@@ -9058,10 +9058,10 @@
         <v>1</v>
       </c>
       <c r="M101" t="n">
-        <v>-58.411053</v>
+        <v>-58.408934</v>
       </c>
       <c r="N101" t="n">
-        <v>-34.618979</v>
+        <v>-34.604273</v>
       </c>
       <c r="O101" t="inlineStr">
         <is>
@@ -9075,7 +9075,7 @@
       </c>
       <c r="Q101" t="inlineStr">
         <is>
-          <t>CEN-J</t>
+          <t>CLI-H</t>
         </is>
       </c>
       <c r="R101" t="inlineStr">
@@ -9087,7 +9087,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>S00379764</t>
+          <t>S00379996</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -9097,7 +9097,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>JAURES JEAN 491</t>
+          <t>SARANDI 1439</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -9112,7 +9112,7 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>813046795</t>
+          <t>813046806</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
@@ -9144,14 +9144,14 @@
         <v>1</v>
       </c>
       <c r="M102" t="n">
-        <v>-58.408934</v>
+        <v>-58.393455</v>
       </c>
       <c r="N102" t="n">
-        <v>-34.604273</v>
+        <v>-34.625779</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P102" t="inlineStr">
@@ -9161,7 +9161,7 @@
       </c>
       <c r="Q102" t="inlineStr">
         <is>
-          <t>CLI-H</t>
+          <t>CON-C</t>
         </is>
       </c>
       <c r="R102" t="inlineStr">
@@ -9173,7 +9173,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>S00379996</t>
+          <t>8823</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -9183,7 +9183,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>SARANDI 1439</t>
+          <t>SARMIENTO 2108</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -9198,7 +9198,7 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>813046806</t>
+          <t>813046819</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
@@ -9230,14 +9230,14 @@
         <v>1</v>
       </c>
       <c r="M103" t="n">
-        <v>-58.393455</v>
+        <v>-58.39675</v>
       </c>
       <c r="N103" t="n">
-        <v>-34.625779</v>
+        <v>-34.605996</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P103" t="inlineStr">
@@ -9247,7 +9247,7 @@
       </c>
       <c r="Q103" t="inlineStr">
         <is>
-          <t>CON-C</t>
+          <t>CLI-B</t>
         </is>
       </c>
       <c r="R103" t="inlineStr">
@@ -9259,7 +9259,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>8823</t>
+          <t>8829</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -9269,12 +9269,12 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>SARMIENTO 2108</t>
+          <t>SANCHEZ DE BUSTAMANTE 633</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -9284,7 +9284,7 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>813046819</t>
+          <t>813046866</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
@@ -9316,10 +9316,10 @@
         <v>1</v>
       </c>
       <c r="M104" t="n">
-        <v>-58.39675</v>
+        <v>-58.414203</v>
       </c>
       <c r="N104" t="n">
-        <v>-34.605996</v>
+        <v>-34.602602</v>
       </c>
       <c r="O104" t="inlineStr">
         <is>
@@ -9333,7 +9333,7 @@
       </c>
       <c r="Q104" t="inlineStr">
         <is>
-          <t>CLI-B</t>
+          <t>CLI-G</t>
         </is>
       </c>
       <c r="R104" t="inlineStr">
@@ -9345,7 +9345,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>8829</t>
+          <t>8846</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -9355,7 +9355,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>SANCHEZ DE BUSTAMANTE 633</t>
+          <t>RIVADAVIA AV 4245</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -9370,7 +9370,7 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>813046866</t>
+          <t>813046970</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
@@ -9402,10 +9402,10 @@
         <v>1</v>
       </c>
       <c r="M105" t="n">
-        <v>-58.414203</v>
+        <v>-58.425567</v>
       </c>
       <c r="N105" t="n">
-        <v>-34.602602</v>
+        <v>-34.613382</v>
       </c>
       <c r="O105" t="inlineStr">
         <is>
@@ -9419,7 +9419,7 @@
       </c>
       <c r="Q105" t="inlineStr">
         <is>
-          <t>CLI-G</t>
+          <t>ALM-D</t>
         </is>
       </c>
       <c r="R105" t="inlineStr">
@@ -9431,7 +9431,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>8846</t>
+          <t>8848</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -9441,7 +9441,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>RIVADAVIA AV 4245</t>
+          <t>DIAZ VELEZ AV 4449</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -9456,7 +9456,7 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>813046970</t>
+          <t>813046971</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
@@ -9488,10 +9488,10 @@
         <v>1</v>
       </c>
       <c r="M106" t="n">
-        <v>-58.425567</v>
+        <v>-58.429714</v>
       </c>
       <c r="N106" t="n">
-        <v>-34.613382</v>
+        <v>-34.608645</v>
       </c>
       <c r="O106" t="inlineStr">
         <is>
@@ -9505,7 +9505,7 @@
       </c>
       <c r="Q106" t="inlineStr">
         <is>
-          <t>ALM-D</t>
+          <t>ALM-K</t>
         </is>
       </c>
       <c r="R106" t="inlineStr">
@@ -9517,7 +9517,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>8848</t>
+          <t>8851</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -9527,7 +9527,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>DIAZ VELEZ AV 4449</t>
+          <t>LAS CASAS 3989</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -9542,7 +9542,7 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>813046971</t>
+          <t>813046994</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
@@ -9574,14 +9574,14 @@
         <v>1</v>
       </c>
       <c r="M107" t="n">
-        <v>-58.429714</v>
+        <v>-58.421676</v>
       </c>
       <c r="N107" t="n">
-        <v>-34.608645</v>
+        <v>-34.635878</v>
       </c>
       <c r="O107" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P107" t="inlineStr">
@@ -9591,7 +9591,7 @@
       </c>
       <c r="Q107" t="inlineStr">
         <is>
-          <t>ALM-K</t>
+          <t>PPT-R</t>
         </is>
       </c>
       <c r="R107" t="inlineStr">
@@ -9603,7 +9603,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>8851</t>
+          <t>8852</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -9613,7 +9613,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>LAS CASAS 3989</t>
+          <t>SALCEDO 3541</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -9628,7 +9628,7 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>813046994</t>
+          <t>813047007</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
@@ -9648,7 +9648,7 @@
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo/Fuente Teco</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
@@ -9660,10 +9660,10 @@
         <v>1</v>
       </c>
       <c r="M108" t="n">
-        <v>-58.421676</v>
+        <v>-58.415121</v>
       </c>
       <c r="N108" t="n">
-        <v>-34.635878</v>
+        <v>-34.633772</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -9677,7 +9677,7 @@
       </c>
       <c r="Q108" t="inlineStr">
         <is>
-          <t>PPT-R</t>
+          <t>PPT-E</t>
         </is>
       </c>
       <c r="R108" t="inlineStr">
@@ -9689,7 +9689,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>8852</t>
+          <t>8853</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -9699,7 +9699,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>SALCEDO 3541</t>
+          <t>TARIJA 4079</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -9714,7 +9714,7 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>813047007</t>
+          <t>813047012</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
@@ -9734,7 +9734,7 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>Nodo/Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
@@ -9746,10 +9746,10 @@
         <v>1</v>
       </c>
       <c r="M109" t="n">
-        <v>-58.415121</v>
+        <v>-58.421804</v>
       </c>
       <c r="N109" t="n">
-        <v>-34.633772</v>
+        <v>-34.629558</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -9763,7 +9763,7 @@
       </c>
       <c r="Q109" t="inlineStr">
         <is>
-          <t>PPT-E</t>
+          <t>PPT-R</t>
         </is>
       </c>
       <c r="R109" t="inlineStr">
@@ -9775,7 +9775,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>8853</t>
+          <t>8854</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -9785,7 +9785,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>TARIJA 4079</t>
+          <t>TIMBUES 2086</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -9800,7 +9800,7 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>813047012</t>
+          <t>813047017</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
@@ -9832,10 +9832,10 @@
         <v>1</v>
       </c>
       <c r="M110" t="n">
-        <v>-58.421804</v>
+        <v>-58.421835</v>
       </c>
       <c r="N110" t="n">
-        <v>-34.629558</v>
+        <v>-34.63863</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -9849,7 +9849,7 @@
       </c>
       <c r="Q110" t="inlineStr">
         <is>
-          <t>PPT-R</t>
+          <t>PPT-L</t>
         </is>
       </c>
       <c r="R110" t="inlineStr">
@@ -9861,7 +9861,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>8854</t>
+          <t>8855</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -9871,7 +9871,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>TIMBUES 2086</t>
+          <t>GOMEZ VALENTIN 3684</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -9886,7 +9886,7 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>813047017</t>
+          <t>813047019</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
@@ -9918,14 +9918,14 @@
         <v>1</v>
       </c>
       <c r="M111" t="n">
-        <v>-58.421835</v>
+        <v>-58.416726</v>
       </c>
       <c r="N111" t="n">
-        <v>-34.63863</v>
+        <v>-34.604773</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P111" t="inlineStr">
@@ -9935,7 +9935,7 @@
       </c>
       <c r="Q111" t="inlineStr">
         <is>
-          <t>PPT-L</t>
+          <t>CLI-K</t>
         </is>
       </c>
       <c r="R111" t="inlineStr">
@@ -9947,7 +9947,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>8855</t>
+          <t>S00390896</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -9957,12 +9957,12 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>GOMEZ VALENTIN 3684</t>
+          <t>AV INDEPENDENCIA 2018</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -9972,7 +9972,7 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>813047019</t>
+          <t>813047657</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
@@ -10004,10 +10004,10 @@
         <v>1</v>
       </c>
       <c r="M112" t="n">
-        <v>-58.416726</v>
+        <v>-58.39469</v>
       </c>
       <c r="N112" t="n">
-        <v>-34.604773</v>
+        <v>-34.618394</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -10021,7 +10021,7 @@
       </c>
       <c r="Q112" t="inlineStr">
         <is>
-          <t>CLI-K</t>
+          <t>CEN-C</t>
         </is>
       </c>
       <c r="R112" t="inlineStr">
@@ -10033,22 +10033,22 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>S00390896</t>
+          <t>RB00001</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>4/11/2026</t>
+          <t>4/20/2026</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>AV INDEPENDENCIA 2018</t>
+          <t>BELGRANO AV. 3715</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -10058,7 +10058,7 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>813047657</t>
+          <t>813304903</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
@@ -10090,10 +10090,10 @@
         <v>1</v>
       </c>
       <c r="M113" t="n">
-        <v>-58.39469</v>
+        <v>-58.418851</v>
       </c>
       <c r="N113" t="n">
-        <v>-34.618394</v>
+        <v>-34.615716</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -10107,7 +10107,7 @@
       </c>
       <c r="Q113" t="inlineStr">
         <is>
-          <t>CEN-C</t>
+          <t>ALM-C</t>
         </is>
       </c>
       <c r="R113" t="inlineStr">
@@ -10119,7 +10119,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>RB00001</t>
+          <t>AM00039</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -10129,7 +10129,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>BELGRANO AV. 3715</t>
+          <t>CASTRO BARROS 852</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -10144,7 +10144,7 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>813304903</t>
+          <t>813304915</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
@@ -10176,14 +10176,14 @@
         <v>1</v>
       </c>
       <c r="M114" t="n">
-        <v>-58.418851</v>
+        <v>-58.419281</v>
       </c>
       <c r="N114" t="n">
-        <v>-34.615716</v>
+        <v>-34.62215</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P114" t="inlineStr">
@@ -10193,7 +10193,7 @@
       </c>
       <c r="Q114" t="inlineStr">
         <is>
-          <t>ALM-C</t>
+          <t>ALM-A</t>
         </is>
       </c>
       <c r="R114" t="inlineStr">
@@ -10205,7 +10205,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>AM00039</t>
+          <t>8940</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -10215,12 +10215,12 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>CASTRO BARROS 852</t>
+          <t>ALSINA, ADOLFO 3293</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -10230,7 +10230,7 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>813304915</t>
+          <t>813350607</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
@@ -10262,14 +10262,14 @@
         <v>1</v>
       </c>
       <c r="M115" t="n">
-        <v>-58.419281</v>
+        <v>-58.412936</v>
       </c>
       <c r="N115" t="n">
-        <v>-34.62215</v>
+        <v>-34.613332</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P115" t="inlineStr">
@@ -10279,7 +10279,7 @@
       </c>
       <c r="Q115" t="inlineStr">
         <is>
-          <t>ALM-A</t>
+          <t>CEN-I</t>
         </is>
       </c>
       <c r="R115" t="inlineStr">
@@ -10291,7 +10291,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>8940</t>
+          <t>S00423738</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -10301,7 +10301,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>ALSINA, ADOLFO 3293</t>
+          <t>CATAMARCA 568</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -10316,7 +10316,7 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>813350607</t>
+          <t>813350620</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
@@ -10348,10 +10348,10 @@
         <v>1</v>
       </c>
       <c r="M116" t="n">
-        <v>-58.412936</v>
+        <v>-58.405541</v>
       </c>
       <c r="N116" t="n">
-        <v>-34.613332</v>
+        <v>-34.616959</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -10365,7 +10365,7 @@
       </c>
       <c r="Q116" t="inlineStr">
         <is>
-          <t>CEN-I</t>
+          <t>CEN-M</t>
         </is>
       </c>
       <c r="R116" t="inlineStr">
@@ -10377,22 +10377,22 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>S00423738</t>
+          <t>S00299569</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>4/20/2026</t>
+          <t>4/21/2026</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>CATAMARCA 568</t>
+          <t>YRIGOYEN, HIPOLITO AV. 4156</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -10402,7 +10402,7 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>813350620</t>
+          <t>813350953</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
@@ -10434,10 +10434,10 @@
         <v>1</v>
       </c>
       <c r="M117" t="n">
-        <v>-58.405541</v>
+        <v>-58.425213</v>
       </c>
       <c r="N117" t="n">
-        <v>-34.616959</v>
+        <v>-34.614924</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -10451,7 +10451,7 @@
       </c>
       <c r="Q117" t="inlineStr">
         <is>
-          <t>CEN-M</t>
+          <t>ALM-D</t>
         </is>
       </c>
       <c r="R117" t="inlineStr">
@@ -10463,7 +10463,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>S00299569</t>
+          <t>S004318770</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -10473,7 +10473,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>YRIGOYEN, HIPOLITO AV. 4156</t>
+          <t>SARMIENTO 4290</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -10488,7 +10488,7 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>813350953</t>
+          <t>813351576</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
@@ -10520,10 +10520,10 @@
         <v>1</v>
       </c>
       <c r="M118" t="n">
-        <v>-58.425213</v>
+        <v>-58.425764</v>
       </c>
       <c r="N118" t="n">
-        <v>-34.614924</v>
+        <v>-34.604359</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
@@ -10537,7 +10537,7 @@
       </c>
       <c r="Q118" t="inlineStr">
         <is>
-          <t>ALM-D</t>
+          <t>ALM-L</t>
         </is>
       </c>
       <c r="R118" t="inlineStr">
@@ -10549,7 +10549,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>S004318770</t>
+          <t>S00431893</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -10559,7 +10559,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>SARMIENTO 4290</t>
+          <t>MUÑIZ 1151</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -10574,7 +10574,7 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>813351576</t>
+          <t>814105853</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
@@ -10606,14 +10606,14 @@
         <v>1</v>
       </c>
       <c r="M119" t="n">
-        <v>-58.425764</v>
+        <v>-58.425442</v>
       </c>
       <c r="N119" t="n">
-        <v>-34.604359</v>
+        <v>-34.627634</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P119" t="inlineStr">
@@ -10623,7 +10623,7 @@
       </c>
       <c r="Q119" t="inlineStr">
         <is>
-          <t>ALM-L</t>
+          <t>PPT-P</t>
         </is>
       </c>
       <c r="R119" t="inlineStr">
@@ -10635,7 +10635,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>S00431893</t>
+          <t>S00434849</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -10645,7 +10645,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>MUÑIZ 1151</t>
+          <t>YRIGOYEN, HIPOLITO AV. 3484</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -10660,7 +10660,7 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>814105853</t>
+          <t>813352212</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
@@ -10692,14 +10692,14 @@
         <v>1</v>
       </c>
       <c r="M120" t="n">
-        <v>-58.425442</v>
+        <v>-58.416028</v>
       </c>
       <c r="N120" t="n">
-        <v>-34.627634</v>
+        <v>-34.613538</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P120" t="inlineStr">
@@ -10709,7 +10709,7 @@
       </c>
       <c r="Q120" t="inlineStr">
         <is>
-          <t>PPT-P</t>
+          <t>CEN-J</t>
         </is>
       </c>
       <c r="R120" t="inlineStr">
@@ -10721,7 +10721,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>S00434849</t>
+          <t xml:space="preserve">9009 </t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -10731,7 +10731,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>YRIGOYEN, HIPOLITO AV. 3484</t>
+          <t>SANCHEZ DE LORIA 1913</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -10746,7 +10746,7 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>813352212</t>
+          <t>813352473</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
@@ -10778,14 +10778,14 @@
         <v>1</v>
       </c>
       <c r="M121" t="n">
-        <v>-58.416028</v>
+        <v>-58.411474</v>
       </c>
       <c r="N121" t="n">
-        <v>-34.613538</v>
+        <v>-34.633143</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P121" t="inlineStr">
@@ -10795,7 +10795,7 @@
       </c>
       <c r="Q121" t="inlineStr">
         <is>
-          <t>CEN-J</t>
+          <t>PPT-Q</t>
         </is>
       </c>
       <c r="R121" t="inlineStr">
@@ -10807,7 +10807,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t xml:space="preserve">9009 </t>
+          <t xml:space="preserve">9011 </t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -10817,7 +10817,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>SANCHEZ DE LORIA 1913</t>
+          <t>SANCHEZ DE LORIA 1583</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -10832,7 +10832,7 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>813352473</t>
+          <t>813352481</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
@@ -10864,14 +10864,14 @@
         <v>1</v>
       </c>
       <c r="M122" t="n">
-        <v>-58.411474</v>
+        <v>-58.411926</v>
       </c>
       <c r="N122" t="n">
-        <v>-34.633143</v>
+        <v>-34.628861</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P122" t="inlineStr">
@@ -10881,7 +10881,7 @@
       </c>
       <c r="Q122" t="inlineStr">
         <is>
-          <t>PPT-Q</t>
+          <t>PPT-E</t>
         </is>
       </c>
       <c r="R122" t="inlineStr">
@@ -10893,7 +10893,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t xml:space="preserve">9011 </t>
+          <t xml:space="preserve">9012 </t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -10903,7 +10903,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>SANCHEZ DE LORIA 1583</t>
+          <t xml:space="preserve">LINIERS VIRREY 2315 </t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -10918,7 +10918,7 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>813352481</t>
+          <t>813352482</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
@@ -10950,14 +10950,14 @@
         <v>1</v>
       </c>
       <c r="M123" t="n">
-        <v>-58.411926</v>
+        <v>-58.41191</v>
       </c>
       <c r="N123" t="n">
-        <v>-34.628861</v>
+        <v>-34.637333</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P123" t="inlineStr">
@@ -10967,7 +10967,7 @@
       </c>
       <c r="Q123" t="inlineStr">
         <is>
-          <t>PPT-E</t>
+          <t>PPT-Q</t>
         </is>
       </c>
       <c r="R123" t="inlineStr">
@@ -10979,7 +10979,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t xml:space="preserve">9012 </t>
+          <t xml:space="preserve">9014 </t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -10989,7 +10989,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t xml:space="preserve">LINIERS VIRREY 2315 </t>
+          <t>LINIERS VIRREY 896</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -11004,7 +11004,7 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>813352482</t>
+          <t>813352486</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
@@ -11036,14 +11036,14 @@
         <v>1</v>
       </c>
       <c r="M124" t="n">
-        <v>-58.41191</v>
+        <v>-58.413645</v>
       </c>
       <c r="N124" t="n">
-        <v>-34.637333</v>
+        <v>-34.621935</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P124" t="inlineStr">
@@ -11053,7 +11053,7 @@
       </c>
       <c r="Q124" t="inlineStr">
         <is>
-          <t>PPT-Q</t>
+          <t>CEN-P</t>
         </is>
       </c>
       <c r="R124" t="inlineStr">
@@ -11065,7 +11065,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t xml:space="preserve">9014 </t>
+          <t xml:space="preserve">9016 </t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -11075,7 +11075,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>LINIERS VIRREY 896</t>
+          <t>HUMBERTO 1° 3368</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -11090,7 +11090,7 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>813352486</t>
+          <t>813352494</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
@@ -11122,10 +11122,10 @@
         <v>1</v>
       </c>
       <c r="M125" t="n">
-        <v>-58.413645</v>
+        <v>-58.413189</v>
       </c>
       <c r="N125" t="n">
-        <v>-34.621935</v>
+        <v>-34.624187</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
@@ -11151,7 +11151,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t xml:space="preserve">9016 </t>
+          <t xml:space="preserve">9017 </t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -11161,7 +11161,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>HUMBERTO 1° 3368</t>
+          <t>MUÑIZ 1237</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -11176,7 +11176,7 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>813352494</t>
+          <t>814105864</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
@@ -11208,10 +11208,10 @@
         <v>1</v>
       </c>
       <c r="M126" t="n">
-        <v>-58.413189</v>
+        <v>-58.425206</v>
       </c>
       <c r="N126" t="n">
-        <v>-34.624187</v>
+        <v>-34.628705</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -11225,7 +11225,7 @@
       </c>
       <c r="Q126" t="inlineStr">
         <is>
-          <t>CEN-P</t>
+          <t>PPT-P</t>
         </is>
       </c>
       <c r="R126" t="inlineStr">
@@ -11237,7 +11237,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t xml:space="preserve">9017 </t>
+          <t xml:space="preserve">9020 </t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -11247,7 +11247,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>MUÑIZ 1237</t>
+          <t>TARIJA 3497</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -11262,7 +11262,7 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>814105864</t>
+          <t>813352497</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
@@ -11294,10 +11294,10 @@
         <v>1</v>
       </c>
       <c r="M127" t="n">
-        <v>-58.425206</v>
+        <v>-58.414424</v>
       </c>
       <c r="N127" t="n">
-        <v>-34.628705</v>
+        <v>-34.628778</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -11311,7 +11311,7 @@
       </c>
       <c r="Q127" t="inlineStr">
         <is>
-          <t>PPT-P</t>
+          <t>PPT-E</t>
         </is>
       </c>
       <c r="R127" t="inlineStr">
@@ -11323,17 +11323,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t xml:space="preserve">9020 </t>
+          <t>9028</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>4/21/2026</t>
+          <t>4/24/2026</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>TARIJA 3497</t>
+          <t>BRAVO, MARIO 740</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -11348,7 +11348,7 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>813352497</t>
+          <t>813352774</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
@@ -11380,14 +11380,14 @@
         <v>1</v>
       </c>
       <c r="M128" t="n">
-        <v>-58.414424</v>
+        <v>-58.416308</v>
       </c>
       <c r="N128" t="n">
-        <v>-34.628778</v>
+        <v>-34.601047</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P128" t="inlineStr">
@@ -11397,7 +11397,7 @@
       </c>
       <c r="Q128" t="inlineStr">
         <is>
-          <t>PPT-E</t>
+          <t>CLI-G</t>
         </is>
       </c>
       <c r="R128" t="inlineStr">
@@ -11409,7 +11409,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>9028</t>
+          <t>S00413025</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -11419,12 +11419,12 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>BRAVO, MARIO 740</t>
+          <t>CHILE 2550</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -11434,7 +11434,7 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>813352774</t>
+          <t>813352855</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
@@ -11466,10 +11466,10 @@
         <v>1</v>
       </c>
       <c r="M129" t="n">
-        <v>-58.416308</v>
+        <v>-58.40174</v>
       </c>
       <c r="N129" t="n">
-        <v>-34.601047</v>
+        <v>-34.617754</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -11483,7 +11483,7 @@
       </c>
       <c r="Q129" t="inlineStr">
         <is>
-          <t>CLI-G</t>
+          <t>CEN-M</t>
         </is>
       </c>
       <c r="R129" t="inlineStr">
@@ -11495,7 +11495,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>S00413025</t>
+          <t>S00429731</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -11505,7 +11505,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>CHILE 2550</t>
+          <t xml:space="preserve">ALSINA, ADOLFO 2291 </t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -11520,7 +11520,7 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>813352855</t>
+          <t>813352873</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
@@ -11552,10 +11552,10 @@
         <v>1</v>
       </c>
       <c r="M130" t="n">
-        <v>-58.40174</v>
+        <v>-58.398771</v>
       </c>
       <c r="N130" t="n">
-        <v>-34.617754</v>
+        <v>-34.611932</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -11569,7 +11569,7 @@
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>CEN-M</t>
+          <t>CEN-G</t>
         </is>
       </c>
       <c r="R130" t="inlineStr">
@@ -11581,22 +11581,22 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>S00429731</t>
+          <t>9046</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>4/24/2026</t>
+          <t>4/29/2026</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t xml:space="preserve">ALSINA, ADOLFO 2291 </t>
+          <t xml:space="preserve">GALLEGOS 3443 </t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -11606,7 +11606,7 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>813352873</t>
+          <t>813353299</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
@@ -11638,14 +11638,14 @@
         <v>1</v>
       </c>
       <c r="M131" t="n">
-        <v>-58.398771</v>
+        <v>-58.413647</v>
       </c>
       <c r="N131" t="n">
-        <v>-34.611932</v>
+        <v>-34.631434</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P131" t="inlineStr">
@@ -11655,7 +11655,7 @@
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>CEN-G</t>
+          <t>PPT-E</t>
         </is>
       </c>
       <c r="R131" t="inlineStr">
@@ -11667,17 +11667,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>9046</t>
+          <t xml:space="preserve">9045 </t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>4/29/2026</t>
+          <t>4/30/2026</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t xml:space="preserve">GALLEGOS 3443 </t>
+          <t>LINIERS VIRREY 1793</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -11692,7 +11692,7 @@
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>813353299</t>
+          <t>813631423</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
@@ -11724,14 +11724,14 @@
         <v>1</v>
       </c>
       <c r="M132" t="n">
-        <v>-58.413647</v>
+        <v>-58.413025</v>
       </c>
       <c r="N132" t="n">
-        <v>-34.631434</v>
+        <v>-34.631929</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P132" t="inlineStr">
@@ -11741,7 +11741,7 @@
       </c>
       <c r="Q132" t="inlineStr">
         <is>
-          <t>PPT-E</t>
+          <t>PPT-Q</t>
         </is>
       </c>
       <c r="R132" t="inlineStr">
@@ -11753,7 +11753,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t xml:space="preserve">9045 </t>
+          <t>9049</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -11763,7 +11763,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>LINIERS VIRREY 1793</t>
+          <t>BATHURST 3377</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -11778,7 +11778,7 @@
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>813631423</t>
+          <t>813631424</t>
         </is>
       </c>
       <c r="G133" t="inlineStr">
@@ -11810,10 +11810,10 @@
         <v>1</v>
       </c>
       <c r="M133" t="n">
-        <v>-58.413025</v>
+        <v>-58.411896</v>
       </c>
       <c r="N133" t="n">
-        <v>-34.631929</v>
+        <v>-34.636028</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -11839,22 +11839,22 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>9049</t>
+          <t>S00215089</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>4/30/2026</t>
+          <t>5/10/2026</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>BATHURST 3377</t>
+          <t>LARREA 122</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
@@ -11864,7 +11864,7 @@
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>813631424</t>
+          <t>813631550</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
@@ -11896,14 +11896,14 @@
         <v>1</v>
       </c>
       <c r="M134" t="n">
-        <v>-58.411896</v>
+        <v>-58.401972</v>
       </c>
       <c r="N134" t="n">
-        <v>-34.636028</v>
+        <v>-34.608317</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P134" t="inlineStr">
@@ -11913,7 +11913,7 @@
       </c>
       <c r="Q134" t="inlineStr">
         <is>
-          <t>PPT-Q</t>
+          <t>CLI-D</t>
         </is>
       </c>
       <c r="R134" t="inlineStr">
@@ -11925,7 +11925,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>S00215089</t>
+          <t>S00401648</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -11935,7 +11935,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>LARREA 122</t>
+          <t>JUNIN 312</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -11950,7 +11950,7 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>813631550</t>
+          <t>813632251</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
@@ -11970,7 +11970,7 @@
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
@@ -11982,10 +11982,10 @@
         <v>1</v>
       </c>
       <c r="M135" t="n">
-        <v>-58.401972</v>
+        <v>-58.396676</v>
       </c>
       <c r="N135" t="n">
-        <v>-34.608317</v>
+        <v>-34.605753</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
@@ -11999,7 +11999,7 @@
       </c>
       <c r="Q135" t="inlineStr">
         <is>
-          <t>CLI-D</t>
+          <t>CLI-B</t>
         </is>
       </c>
       <c r="R135" t="inlineStr">
@@ -12011,7 +12011,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>S00401648</t>
+          <t>S00465940</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -12021,12 +12021,12 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>JUNIN 312</t>
+          <t>BELGRANO AV. 3669</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
@@ -12036,7 +12036,7 @@
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>813632251</t>
+          <t>813632257</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
@@ -12056,7 +12056,7 @@
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
@@ -12068,10 +12068,10 @@
         <v>1</v>
       </c>
       <c r="M136" t="n">
-        <v>-58.396676</v>
+        <v>-58.417949</v>
       </c>
       <c r="N136" t="n">
-        <v>-34.605753</v>
+        <v>-34.615674</v>
       </c>
       <c r="O136" t="inlineStr">
         <is>
@@ -12085,7 +12085,7 @@
       </c>
       <c r="Q136" t="inlineStr">
         <is>
-          <t>CLI-B</t>
+          <t>ALM-C</t>
         </is>
       </c>
       <c r="R136" t="inlineStr">
@@ -12097,7 +12097,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>S00465940</t>
+          <t>9113</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -12107,12 +12107,12 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>BELGRANO AV. 3669</t>
+          <t>JAURES, JEAN 309</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
@@ -12122,7 +12122,7 @@
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>813632257</t>
+          <t>813632439</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
@@ -12154,10 +12154,10 @@
         <v>1</v>
       </c>
       <c r="M137" t="n">
-        <v>-58.417949</v>
+        <v>-58.409868</v>
       </c>
       <c r="N137" t="n">
-        <v>-34.615674</v>
+        <v>-34.606562</v>
       </c>
       <c r="O137" t="inlineStr">
         <is>
@@ -12171,7 +12171,7 @@
       </c>
       <c r="Q137" t="inlineStr">
         <is>
-          <t>ALM-C</t>
+          <t>CLI-H</t>
         </is>
       </c>
       <c r="R137" t="inlineStr">
@@ -12183,22 +12183,22 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>9113</t>
+          <t>S00364775</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>5/10/2026</t>
+          <t>5/13/2026</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>JAURES, JEAN 309</t>
+          <t>CASTRO 511</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
@@ -12206,11 +12206,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F138" t="inlineStr">
-        <is>
-          <t>813632439</t>
-        </is>
-      </c>
+      <c r="F138" t="inlineStr"/>
       <c r="G138" t="inlineStr">
         <is>
           <t>FIBERWORK</t>
@@ -12218,12 +12214,12 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>NORMALIZAR RIENDA A PIQUE</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Tensor</t>
         </is>
       </c>
       <c r="J138" t="inlineStr">
@@ -12233,17 +12229,17 @@
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L138" t="n">
         <v>1</v>
       </c>
       <c r="M138" t="n">
-        <v>-58.409868</v>
+        <v>-58.420597</v>
       </c>
       <c r="N138" t="n">
-        <v>-34.606562</v>
+        <v>-34.617818</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -12257,7 +12253,7 @@
       </c>
       <c r="Q138" t="inlineStr">
         <is>
-          <t>CLI-H</t>
+          <t>ALM-B</t>
         </is>
       </c>
       <c r="R138" t="inlineStr">
@@ -12269,7 +12265,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>S00364775</t>
+          <t>S00493114</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -12279,12 +12275,12 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>CASTRO 511</t>
+          <t>ARENALES 3648</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
@@ -12292,7 +12288,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F139" t="inlineStr"/>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>813352547</t>
+        </is>
+      </c>
       <c r="G139" t="inlineStr">
         <is>
           <t>FIBERWORK</t>
@@ -12300,36 +12300,36 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>NORMALIZAR RIENDA A PIQUE</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>Tensor</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L139" t="n">
         <v>1</v>
       </c>
       <c r="M139" t="n">
-        <v>-58.420597</v>
+        <v>-58.413656</v>
       </c>
       <c r="N139" t="n">
-        <v>-34.617818</v>
+        <v>-34.585464</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P139" t="inlineStr">
@@ -12339,7 +12339,7 @@
       </c>
       <c r="Q139" t="inlineStr">
         <is>
-          <t>ALM-B</t>
+          <t>AGU-L</t>
         </is>
       </c>
       <c r="R139" t="inlineStr">
@@ -12351,7 +12351,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>S00493114</t>
+          <t xml:space="preserve">7880 </t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -12361,12 +12361,12 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>ARENALES 3648</t>
+          <t>MUÑIZ 16</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
@@ -12376,7 +12376,7 @@
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>813352547</t>
+          <t>814109709</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
@@ -12396,7 +12396,7 @@
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -12408,14 +12408,14 @@
         <v>1</v>
       </c>
       <c r="M140" t="n">
-        <v>-58.413656</v>
+        <v>-58.427498</v>
       </c>
       <c r="N140" t="n">
-        <v>-34.585464</v>
+        <v>-34.614599</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P140" t="inlineStr">
@@ -12425,7 +12425,7 @@
       </c>
       <c r="Q140" t="inlineStr">
         <is>
-          <t>AGU-L</t>
+          <t>ALM-D</t>
         </is>
       </c>
       <c r="R140" t="inlineStr">
@@ -12437,7 +12437,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t xml:space="preserve">7880 </t>
+          <t xml:space="preserve">9923 </t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -12447,7 +12447,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>MUÑIZ 16</t>
+          <t>PRINGLES 1094</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -12462,7 +12462,7 @@
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>814109709</t>
+          <t>814109753</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
@@ -12494,10 +12494,10 @@
         <v>1</v>
       </c>
       <c r="M141" t="n">
-        <v>-58.427498</v>
+        <v>-58.426722</v>
       </c>
       <c r="N141" t="n">
-        <v>-34.614599</v>
+        <v>-34.599427</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -12511,7 +12511,7 @@
       </c>
       <c r="Q141" t="inlineStr">
         <is>
-          <t>ALM-D</t>
+          <t>CLI-M</t>
         </is>
       </c>
       <c r="R141" t="inlineStr">
@@ -12523,17 +12523,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t xml:space="preserve">9923 </t>
+          <t xml:space="preserve">9019 </t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>5/13/2026</t>
+          <t>5/14/2026</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>PRINGLES 1094</t>
+          <t>CASTRO BARROS AV. 338</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -12548,7 +12548,7 @@
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>814109753</t>
+          <t>814108068</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
@@ -12580,10 +12580,10 @@
         <v>1</v>
       </c>
       <c r="M142" t="n">
-        <v>-58.426722</v>
+        <v>-58.419864</v>
       </c>
       <c r="N142" t="n">
-        <v>-34.599427</v>
+        <v>-34.616375</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -12597,7 +12597,7 @@
       </c>
       <c r="Q142" t="inlineStr">
         <is>
-          <t>CLI-M</t>
+          <t>ALM-C</t>
         </is>
       </c>
       <c r="R142" t="inlineStr">
@@ -12609,7 +12609,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t xml:space="preserve">9019 </t>
+          <t xml:space="preserve">9031 </t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -12619,12 +12619,12 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>CASTRO BARROS AV. 338</t>
+          <t>YRIGOYEN, HIPOLITO 1938</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
@@ -12632,11 +12632,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F143" t="inlineStr">
-        <is>
-          <t>814108068</t>
-        </is>
-      </c>
+      <c r="F143" t="inlineStr"/>
       <c r="G143" t="inlineStr">
         <is>
           <t>FIBERWORK</t>
@@ -12654,7 +12650,7 @@
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo/Fuente Teco</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
@@ -12666,10 +12662,10 @@
         <v>1</v>
       </c>
       <c r="M143" t="n">
-        <v>-58.419864</v>
+        <v>-58.394079</v>
       </c>
       <c r="N143" t="n">
-        <v>-34.616375</v>
+        <v>-34.61051</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -12683,7 +12679,7 @@
       </c>
       <c r="Q143" t="inlineStr">
         <is>
-          <t>ALM-C</t>
+          <t>CEN-G</t>
         </is>
       </c>
       <c r="R143" t="inlineStr">
@@ -12695,7 +12691,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t xml:space="preserve">9031 </t>
+          <t xml:space="preserve">9088 </t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -12705,12 +12701,12 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>YRIGOYEN, HIPOLITO 1938</t>
+          <t>HUMAHUACA 4296</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
@@ -12718,7 +12714,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F144" t="inlineStr"/>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>814108086</t>
+        </is>
+      </c>
       <c r="G144" t="inlineStr">
         <is>
           <t>FIBERWORK</t>
@@ -12736,7 +12736,7 @@
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>Nodo/Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
@@ -12748,10 +12748,10 @@
         <v>1</v>
       </c>
       <c r="M144" t="n">
-        <v>-58.394079</v>
+        <v>-58.425282</v>
       </c>
       <c r="N144" t="n">
-        <v>-34.61051</v>
+        <v>-34.601504</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -12765,7 +12765,7 @@
       </c>
       <c r="Q144" t="inlineStr">
         <is>
-          <t>CEN-G</t>
+          <t>CLI-M</t>
         </is>
       </c>
       <c r="R144" t="inlineStr">
@@ -12777,7 +12777,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t xml:space="preserve">9088 </t>
+          <t xml:space="preserve">10059 </t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -12787,12 +12787,12 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>HUMAHUACA 4296</t>
+          <t xml:space="preserve">SALGUERO, JERONIMO 2296 </t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
@@ -12802,7 +12802,7 @@
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>814108086</t>
+          <t>814111727</t>
         </is>
       </c>
       <c r="G145" t="inlineStr">
@@ -12812,7 +12812,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -12834,14 +12834,14 @@
         <v>1</v>
       </c>
       <c r="M145" t="n">
-        <v>-58.425282</v>
+        <v>-58.411132</v>
       </c>
       <c r="N145" t="n">
-        <v>-34.601504</v>
+        <v>-34.585267</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P145" t="inlineStr">
@@ -12851,7 +12851,7 @@
       </c>
       <c r="Q145" t="inlineStr">
         <is>
-          <t>CLI-M</t>
+          <t>AGU-K</t>
         </is>
       </c>
       <c r="R145" t="inlineStr">
@@ -12863,17 +12863,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t xml:space="preserve">10059 </t>
+          <t>-776</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>5/14/2026</t>
+          <t>6/2/2026</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t xml:space="preserve">SALGUERO, JERONIMO 2296 </t>
+          <t>ALSINA, ADOLFO 2457</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -12888,7 +12888,7 @@
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>814111727</t>
+          <t>814125554</t>
         </is>
       </c>
       <c r="G146" t="inlineStr">
@@ -12898,7 +12898,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -12920,14 +12920,14 @@
         <v>1</v>
       </c>
       <c r="M146" t="n">
-        <v>-58.411132</v>
+        <v>-58.401052</v>
       </c>
       <c r="N146" t="n">
-        <v>-34.585267</v>
+        <v>-34.612103</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P146" t="inlineStr">
@@ -12937,7 +12937,7 @@
       </c>
       <c r="Q146" t="inlineStr">
         <is>
-          <t>AGU-K</t>
+          <t>CEN-H</t>
         </is>
       </c>
       <c r="R146" t="inlineStr">
@@ -12949,7 +12949,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>-776</t>
+          <t>-801</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -12959,7 +12959,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>ALSINA, ADOLFO 2457</t>
+          <t>YRIGOYEN, HIPOLITO 2754</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -12974,7 +12974,7 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>814125554</t>
+          <t>814125643</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
@@ -13006,10 +13006,10 @@
         <v>1</v>
       </c>
       <c r="M147" t="n">
-        <v>-58.401052</v>
+        <v>-58.405116</v>
       </c>
       <c r="N147" t="n">
-        <v>-34.612103</v>
+        <v>-34.611253</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -13035,7 +13035,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>-801</t>
+          <t>-810</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -13045,7 +13045,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>YRIGOYEN, HIPOLITO 2754</t>
+          <t>MEXICO 2183</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -13060,7 +13060,7 @@
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>814125643</t>
+          <t>814125664</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
@@ -13092,10 +13092,10 @@
         <v>1</v>
       </c>
       <c r="M148" t="n">
-        <v>-58.405116</v>
+        <v>-58.397489</v>
       </c>
       <c r="N148" t="n">
-        <v>-34.611253</v>
+        <v>-34.616089</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -13109,7 +13109,7 @@
       </c>
       <c r="Q148" t="inlineStr">
         <is>
-          <t>CEN-H</t>
+          <t>CEN-C</t>
         </is>
       </c>
       <c r="R148" t="inlineStr">
@@ -13121,7 +13121,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>-810</t>
+          <t>-818</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -13131,12 +13131,12 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>MEXICO 2183</t>
+          <t>PRINGLES 795</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
@@ -13146,7 +13146,7 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>814125664</t>
+          <t>814125690</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
@@ -13156,7 +13156,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>base podrida</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -13178,10 +13178,10 @@
         <v>1</v>
       </c>
       <c r="M149" t="n">
-        <v>-58.397489</v>
+        <v>-58.427096</v>
       </c>
       <c r="N149" t="n">
-        <v>-34.616089</v>
+        <v>-34.602833</v>
       </c>
       <c r="O149" t="inlineStr">
         <is>
@@ -13195,7 +13195,7 @@
       </c>
       <c r="Q149" t="inlineStr">
         <is>
-          <t>CEN-C</t>
+          <t>CLI-M</t>
         </is>
       </c>
       <c r="R149" t="inlineStr">
@@ -13207,7 +13207,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>-818</t>
+          <t>-820</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -13217,12 +13217,12 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>PRINGLES 795</t>
+          <t>RIOBAMBA 558</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
@@ -13232,7 +13232,7 @@
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>814125690</t>
+          <t>814125697</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
@@ -13242,7 +13242,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>base podrida</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
@@ -13264,10 +13264,10 @@
         <v>1</v>
       </c>
       <c r="M150" t="n">
-        <v>-58.427096</v>
+        <v>-58.394106</v>
       </c>
       <c r="N150" t="n">
-        <v>-34.602833</v>
+        <v>-34.602514</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -13281,19 +13281,19 @@
       </c>
       <c r="Q150" t="inlineStr">
         <is>
-          <t>CLI-M</t>
+          <t>RET-J</t>
         </is>
       </c>
       <c r="R150" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.1RET</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>-820</t>
+          <t>-828</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -13303,7 +13303,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>RIOBAMBA 558</t>
+          <t>TUCUMAN 2074</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -13318,7 +13318,7 @@
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>814125697</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
@@ -13338,7 +13338,7 @@
       </c>
       <c r="J151" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K151" t="inlineStr">
@@ -13350,10 +13350,10 @@
         <v>1</v>
       </c>
       <c r="M151" t="n">
-        <v>-58.394106</v>
+        <v>-58.396631</v>
       </c>
       <c r="N151" t="n">
-        <v>-34.602514</v>
+        <v>-34.60222</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
@@ -13371,92 +13371,6 @@
         </is>
       </c>
       <c r="R151" t="inlineStr">
-        <is>
-          <t>ARATO-25058.PO.1RET</t>
-        </is>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" t="inlineStr">
-        <is>
-          <t>-828</t>
-        </is>
-      </c>
-      <c r="B152" t="inlineStr">
-        <is>
-          <t>6/2/2026</t>
-        </is>
-      </c>
-      <c r="C152" t="inlineStr">
-        <is>
-          <t>TUCUMAN 2074</t>
-        </is>
-      </c>
-      <c r="D152" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E152" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F152" t="inlineStr">
-        <is>
-          <t>Pendiente ADM</t>
-        </is>
-      </c>
-      <c r="G152" t="inlineStr">
-        <is>
-          <t>FIBERWORK</t>
-        </is>
-      </c>
-      <c r="H152" t="inlineStr">
-        <is>
-          <t>base corroida</t>
-        </is>
-      </c>
-      <c r="I152" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J152" t="inlineStr">
-        <is>
-          <t>Nodo Teco</t>
-        </is>
-      </c>
-      <c r="K152" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L152" t="n">
-        <v>1</v>
-      </c>
-      <c r="M152" t="n">
-        <v>-58.396631</v>
-      </c>
-      <c r="N152" t="n">
-        <v>-34.60222</v>
-      </c>
-      <c r="O152" t="inlineStr">
-        <is>
-          <t>Almagro</t>
-        </is>
-      </c>
-      <c r="P152" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q152" t="inlineStr">
-        <is>
-          <t>RET-J</t>
-        </is>
-      </c>
-      <c r="R152" t="inlineStr">
         <is>
           <t>ARATO-25058.PO.1RET</t>
         </is>

</xml_diff>